<commit_message>
data update for manuscripts submission
</commit_message>
<xml_diff>
--- a/data_raw/country_corrections.xlsx
+++ b/data_raw/country_corrections.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCASTRO\Documents\GitHub\Third-Sector-Size-and-Political-Polarization\data_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCASTRO\Documents\GitHub\Third Sector Size and Resilience\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17BC5C97-F1C8-4C7E-B303-70594F5BDC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFF7FA29-ED00-4C60-B387-9EF85A1A72AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C9FE928A-5FE8-49B9-8D87-397F4059AF5C}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{C9FE928A-5FE8-49B9-8D87-397F4059AF5C}"/>
   </bookViews>
   <sheets>
     <sheet name="country_corrections" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'country_corrections'!$A$1:$B$93</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'country_corrections'!$A$1:$B$103</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="149">
   <si>
     <t>original</t>
   </si>
@@ -448,6 +448,36 @@
   </si>
   <si>
     <t>Antigua and Barbuda</t>
+  </si>
+  <si>
+    <t>Bolivia, Plurinational State of</t>
+  </si>
+  <si>
+    <t>Congo, the Democratic Republic of the</t>
+  </si>
+  <si>
+    <t>Micronesia, Federated States of</t>
+  </si>
+  <si>
+    <t>Iran, Islamic Republic of</t>
+  </si>
+  <si>
+    <t>Korea, Democratic People's Republic of</t>
+  </si>
+  <si>
+    <t>Korea, Republic of</t>
+  </si>
+  <si>
+    <t>Moldova, Republic of</t>
+  </si>
+  <si>
+    <t>Palestine, State of</t>
+  </si>
+  <si>
+    <t>Eswatini, the Kingdom of</t>
+  </si>
+  <si>
+    <t>Tanzania, United Republic of</t>
   </si>
 </sst>
 </file>
@@ -914,8 +944,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -997,8 +1028,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F5C799E2-D7CE-4B96-BB33-F840BFB22CA5}" name="country_corrections" displayName="country_corrections" ref="A1:B93" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:B93" xr:uid="{F5C799E2-D7CE-4B96-BB33-F840BFB22CA5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F5C799E2-D7CE-4B96-BB33-F840BFB22CA5}" name="country_corrections" displayName="country_corrections" ref="A1:B103" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:B103" xr:uid="{F5C799E2-D7CE-4B96-BB33-F840BFB22CA5}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B103">
+    <sortCondition ref="A1:A103"/>
+  </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F28AC23F-6346-4D25-9BF4-F1FCEBC95289}" uniqueName="1" name="original" queryTableFieldId="1" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{109E5AF7-294B-41F2-8D59-658478BD4B60}" uniqueName="2" name=" corrected" queryTableFieldId="2" dataDxfId="0"/>
@@ -1324,7 +1358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED12B22A-9E95-401C-9AC4-F248AB7C779A}">
-  <dimension ref="A1:B93"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="37.26953125" bestFit="1" customWidth="1"/>
@@ -1357,17 +1391,17 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1397,26 +1431,26 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
@@ -1429,7 +1463,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>108</v>
@@ -1437,7 +1471,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
         <v>108</v>
@@ -1452,202 +1486,202 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>13</v>
+      <c r="A16" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>112</v>
+      <c r="A26" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>90</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="B29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="B31" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>93</v>
-      </c>
-      <c r="B35" t="s">
-        <v>116</v>
+      <c r="A35" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B36" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B39" t="s">
-        <v>117</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
-        <v>95</v>
-      </c>
-      <c r="B40" t="s">
+      <c r="A40" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1660,35 +1694,35 @@
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>36</v>
-      </c>
-      <c r="B42" t="s">
+      <c r="A42" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B43" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.45">
@@ -1701,18 +1735,18 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B47" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B48" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.45">
@@ -1725,354 +1759,434 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B50" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="B51" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
-        <v>44</v>
-      </c>
-      <c r="B52" t="s">
-        <v>121</v>
+      <c r="A52" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
-        <v>47</v>
-      </c>
-      <c r="B53" t="s">
-        <v>122</v>
+      <c r="A53" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B54" t="s">
-        <v>122</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B55" t="s">
-        <v>49</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B56" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B57" t="s">
-        <v>123</v>
+        <v>50</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B58" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
-        <v>46</v>
+      <c r="A59" s="1" t="s">
+        <v>146</v>
       </c>
       <c r="B59" t="s">
-        <v>45</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>45</v>
+        <v>107</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="B61" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B62" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B63" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>13</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="B65" t="s">
-        <v>127</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="B66" t="s">
-        <v>128</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B67" t="s">
-        <v>128</v>
+        <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B68" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="B69" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B70" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B71" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B72" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B73" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B74" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B75" t="s">
-        <v>75</v>
+        <v>131</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B76" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B77" t="s">
-        <v>72</v>
+        <v>130</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="B78" t="s">
-        <v>72</v>
+        <v>118</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B79" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B80" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B81" t="s">
-        <v>68</v>
+        <v>133</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B82" t="s">
-        <v>135</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A83" t="s">
-        <v>77</v>
-      </c>
-      <c r="B83" t="s">
-        <v>98</v>
+      <c r="A83" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="B84" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="B85" t="s">
-        <v>98</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="B86" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="B87" t="s">
-        <v>136</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="B88" t="s">
-        <v>136</v>
+        <v>72</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B89" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="B90" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B91" t="s">
-        <v>83</v>
+        <v>134</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="B92" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
+        <v>75</v>
+      </c>
+      <c r="B93" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A94" t="s">
+        <v>76</v>
+      </c>
+      <c r="B94" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A95" t="s">
+        <v>77</v>
+      </c>
+      <c r="B95" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A96" t="s">
+        <v>78</v>
+      </c>
+      <c r="B96" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A97" t="s">
         <v>86</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B97" t="s">
         <v>135</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A98" t="s">
+        <v>80</v>
+      </c>
+      <c r="B98" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A99" t="s">
+        <v>100</v>
+      </c>
+      <c r="B99" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A100" t="s">
+        <v>82</v>
+      </c>
+      <c r="B100" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A101" t="s">
+        <v>81</v>
+      </c>
+      <c r="B101" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A102" t="s">
+        <v>52</v>
+      </c>
+      <c r="B102" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A103" t="s">
+        <v>101</v>
+      </c>
+      <c r="B103" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>